<commit_message>
WBC MT v4: documented R5 note on Cover (flat-payout 30.03 superseded by CET1-binding 30.28)
</commit_message>
<xml_diff>
--- a/analyses/wbc/valuations/wbc_muddle_through_valuation_v4_formulas.xlsx
+++ b/analyses/wbc/valuations/wbc_muddle_through_valuation_v4_formulas.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="169" formatCode="#,##0;(#,##0)"/>
     <numFmt numFmtId="170" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,8 +92,15 @@
       <color rgb="00595959"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00833C00"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +131,11 @@
         <bgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -151,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -197,6 +209,12 @@
     <xf numFmtId="170" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -562,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -661,6 +679,41 @@
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>• Trace any output back to inputs by clicking the cell and viewing the formula bar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>Payout convention — superseded note (R5, 25 June 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="44" t="inlineStr">
+        <is>
+          <t>This workbook applies a FLAT 75% dividend payout every year — a simplification — which produces the AUD 30.03 headline above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="44" t="inlineStr">
+        <is>
+          <t>The sounder methodology for a financial institution is the §15.5 CET1-binding payout (the payout flexes down to maintain the CET1 target, returning surplus above buffer). That mechanic is implemented in wbc_scenarios_comparison_v2.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>Canonical WBC Muddle Through under the binding mechanic: AUD 30.28 (~0.8% above this workbook). That is the production bank-engine acceptance number (engine plan R5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="44" t="inlineStr">
+        <is>
+          <t>Decision: Stephen, 25 June 2026 — the CET1-binding mechanic is the methodology for financial institutions. This flat-payout build is retained as a simplified earlier artefact only.</t>
         </is>
       </c>
     </row>

</xml_diff>